<commit_message>
docs: add emojis to the BSCS Year 1 and Precalculus Subject Plans - prefix each Subject Plan name in both shaping TSVs with an emoji, as the other review sets do - regenerate both target-shape workbooks with the builder; the Year root title is now "🖥️ BS Computer Science — 1st Year" and the optional root "📈 Precalculus (Algebra and Trigonometry)" - descriptions unchanged; counts unchanged (218 rows: 50 Reuse / 163 New / 5 Excluded; Precalculus 31 New)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/curriculum/bscs-precalculus-preparatory-target-shape.xlsx
+++ b/docs/curriculum/bscs-precalculus-preparatory-target-shape.xlsx
@@ -525,7 +525,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry) — target shape</t>
+          <t>📈 Precalculus (Algebra and Trigonometry) — target shape</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
@@ -814,7 +814,7 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -2122,7 +2122,7 @@
       <c r="C6" s="6" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -2147,7 +2147,7 @@
       <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2172,7 +2172,7 @@
       <c r="C8" s="6" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -2197,7 +2197,7 @@
       <c r="C9" s="6" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -2222,7 +2222,7 @@
       <c r="C10" s="6" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -2247,7 +2247,7 @@
       <c r="C11" s="6" t="inlineStr"/>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -2272,7 +2272,7 @@
       <c r="C12" s="6" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -2297,7 +2297,7 @@
       <c r="C13" s="6" t="inlineStr"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -2322,7 +2322,7 @@
       <c r="C14" s="6" t="inlineStr"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -2347,7 +2347,7 @@
       <c r="C15" s="6" t="inlineStr"/>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -2372,7 +2372,7 @@
       <c r="C16" s="6" t="inlineStr"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -2397,7 +2397,7 @@
       <c r="C17" s="6" t="inlineStr"/>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -2422,7 +2422,7 @@
       <c r="C18" s="6" t="inlineStr"/>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -2447,7 +2447,7 @@
       <c r="C19" s="6" t="inlineStr"/>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -2472,7 +2472,7 @@
       <c r="C20" s="6" t="inlineStr"/>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -2497,7 +2497,7 @@
       <c r="C21" s="6" t="inlineStr"/>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -2522,7 +2522,7 @@
       <c r="C22" s="6" t="inlineStr"/>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -2582,7 +2582,7 @@
       <c r="C25" s="6" t="inlineStr"/>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -2607,7 +2607,7 @@
       <c r="C26" s="6" t="inlineStr"/>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -2632,7 +2632,7 @@
       <c r="C27" s="6" t="inlineStr"/>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2657,7 +2657,7 @@
       <c r="C28" s="6" t="inlineStr"/>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2682,7 +2682,7 @@
       <c r="C29" s="6" t="inlineStr"/>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -2707,7 +2707,7 @@
       <c r="C30" s="6" t="inlineStr"/>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -2732,7 +2732,7 @@
       <c r="C31" s="6" t="inlineStr"/>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -2792,7 +2792,7 @@
       <c r="C34" s="6" t="inlineStr"/>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2817,7 +2817,7 @@
       <c r="C35" s="6" t="inlineStr"/>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -2842,7 +2842,7 @@
       <c r="C36" s="6" t="inlineStr"/>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2867,7 +2867,7 @@
       <c r="C37" s="6" t="inlineStr"/>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Precalculus (Algebra and Trigonometry)</t>
+          <t>📈 Precalculus (Algebra and Trigonometry)</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">

</xml_diff>